<commit_message>
Allow numeric PKs with FK-parent structural evidence (2D.3).
Accept integer identifiers when referenced by an FK without labeling SURROGATE, and keep accidentally unique Qty rejected.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/workbooks/relationships/rel_integer_unique_not_surrogate.xlsx
+++ b/tests/fixtures/workbooks/relationships/rel_integer_unique_not_surrogate.xlsx
@@ -423,7 +423,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RowNum</t>
+          <t>Qty</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -434,7 +434,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -444,7 +444,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -454,7 +454,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -464,7 +464,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>

</xml_diff>